<commit_message>
New member for fgDeGender
</commit_message>
<xml_diff>
--- a/JSON/fgDeGender_Trefwoorden.xlsx
+++ b/JSON/fgDeGender_Trefwoorden.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo-Club-Hub/JSON/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/JSON/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F80F5D-5DA1-E64A-8455-8FFBF795BAB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AE53E2E-2252-BC49-A2AF-9901634C39C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16640" xr2:uid="{186BA102-7DEB-D04F-9935-E140A076FA03}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{186BA102-7DEB-D04F-9935-E140A076FA03}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabel" sheetId="1" r:id="rId1"/>
@@ -37,10 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="80">
-  <si>
-    <t>Albert</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="80">
   <si>
     <t>Experimenteel</t>
   </si>
@@ -237,9 +234,6 @@
     <t>Museum</t>
   </si>
   <si>
-    <t>Koning</t>
-  </si>
-  <si>
     <t>Zelfexpressie</t>
   </si>
   <si>
@@ -277,6 +271,12 @@
   </si>
   <si>
     <t>Natuur</t>
+  </si>
+  <si>
+    <t>Jos</t>
+  </si>
+  <si>
+    <t>Verhoosel</t>
   </si>
 </sst>
 </file>
@@ -376,7 +376,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -395,12 +395,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -414,7 +408,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -453,12 +447,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="45"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="45"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="45"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -478,8 +466,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -490,9 +478,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -999,12 +984,6 @@
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="13" formatCode="0%"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1664,7 +1643,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A5D2FC80-7473-CB42-8074-67FE4C691AF2}" type="CELLRANGE">
+                    <a:fld id="{6734B8BD-74F3-124A-9E72-E6EA2DA5C473}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1697,7 +1676,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C2E42C5F-182E-AD40-85CB-31C81EA1640B}" type="CELLRANGE">
+                    <a:fld id="{B575EEA0-7261-1C4D-977C-C5BF65721F37}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1731,7 +1710,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{148AAC6F-81F8-E44C-8A94-A1C8747D0350}" type="CELLRANGE">
+                    <a:fld id="{97BAC1A7-27CA-8A45-B9B3-D10E544C8646}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1765,7 +1744,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9B6F0712-144F-7F41-AE44-FA60DF3A8268}" type="CELLRANGE">
+                    <a:fld id="{F69B36BC-18D6-6546-8B5F-232B79EF81AD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1799,7 +1778,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{56EA6538-15B9-3542-B2C1-4FA9211E2065}" type="CELLRANGE">
+                    <a:fld id="{2B6DF37C-0ED7-CF4A-A27E-70FD356A6826}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1833,7 +1812,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DCC46678-2FAF-CD4A-A6DA-C073994EE7CF}" type="CELLRANGE">
+                    <a:fld id="{6525DF71-EEED-CC4E-8296-14A1EA221BA6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1867,7 +1846,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4C2F64B8-1E41-E447-9715-728D08E8F179}" type="CELLRANGE">
+                    <a:fld id="{A396B2AF-9238-6542-AB60-1BFE25A4EACD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1901,7 +1880,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2E18151D-799B-1E42-A21E-ABE3BD4DC279}" type="CELLRANGE">
+                    <a:fld id="{A8806813-E15E-3949-B037-8D211999C198}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1935,7 +1914,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{ECBD3A9E-1332-6B4A-9634-D6294B0EB6F4}" type="CELLRANGE">
+                    <a:fld id="{BA399F62-5741-3041-8D27-5A8CF0AF2BD3}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1969,7 +1948,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E3C5B180-0966-544C-B23F-3F9ED57E332A}" type="CELLRANGE">
+                    <a:fld id="{F907CADB-7B64-A041-97AB-5DEE9A6DF784}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2003,7 +1982,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{ED7A8BAE-EF0B-754B-A879-E9A05FE718F7}" type="CELLRANGE">
+                    <a:fld id="{C20C97D3-4444-C440-B3D6-3B180680CF59}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2037,7 +2016,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7FCDB845-F912-2C4F-885E-A1902B424542}" type="CELLRANGE">
+                    <a:fld id="{9140C00D-ABC1-9A4B-B3E9-484A0AC62DBF}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2071,7 +2050,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{63FB506C-8269-E74E-9A04-91F6A375AEF6}" type="CELLRANGE">
+                    <a:fld id="{FC31CE86-CC40-334F-BCAF-D52B8C15796C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2105,7 +2084,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{44A222D0-4F00-A04A-B97B-59267CC0F4F5}" type="CELLRANGE">
+                    <a:fld id="{86465731-4576-974F-81EB-38D32A248413}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2139,7 +2118,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6C95A3F0-D401-E941-9DB2-BCE197389944}" type="CELLRANGE">
+                    <a:fld id="{AF971FAF-CB21-1646-8A34-1043FC030D4A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2173,7 +2152,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EA6B6C8F-AB81-084D-A125-CC6BEA991A0E}" type="CELLRANGE">
+                    <a:fld id="{C0426F27-5F8B-E545-A6EE-687375523984}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2207,7 +2186,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{21F8FF27-CEEE-C34E-B9B8-A6B78BEBBA50}" type="CELLRANGE">
+                    <a:fld id="{D1885CCF-CAD9-6441-B0B9-A952F9A2C2A1}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2241,7 +2220,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{64D488CF-5C05-C646-BC59-CE4BE09B72DE}" type="CELLRANGE">
+                    <a:fld id="{A5CE89D3-8402-8746-A4E4-1AB087D2BD06}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2275,7 +2254,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8ED2F28C-6DA3-7F4D-B730-5D9E3AC407E7}" type="CELLRANGE">
+                    <a:fld id="{26FF9044-026B-B043-8663-DC5C20724287}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2309,7 +2288,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EB92A9AB-9BF2-4A46-9A6D-B379C321EC38}" type="CELLRANGE">
+                    <a:fld id="{481A5D2F-52DE-C744-A2DE-2C5EB9F4D05B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2343,7 +2322,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9793AE83-7FDE-BA4D-A5D2-2C63C0784255}" type="CELLRANGE">
+                    <a:fld id="{90A10C5B-2B7E-C04B-A534-DE43E35B3F60}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2377,7 +2356,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F5ECEA48-65D1-B54C-9AEC-977F9A05BE5E}" type="CELLRANGE">
+                    <a:fld id="{95C9A821-9216-CB4B-AAAC-74EF09F69EF6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2411,7 +2390,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{04E51CD1-9EB8-904E-93A0-EF1C0BB7266E}" type="CELLRANGE">
+                    <a:fld id="{188A3380-01F8-894A-BFEC-FA2A7DED3AAD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2445,7 +2424,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6DA824D8-21AB-2841-AE41-2C4A0E75DE64}" type="CELLRANGE">
+                    <a:fld id="{D7C1390F-9EC7-DE47-895D-FDA125CA6EBD}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2577,7 +2556,7 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>0</c:v>
@@ -2595,7 +2574,7 @@
                   <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
@@ -3870,103 +3849,103 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" s="2" customFormat="1" ht="127" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="B1" s="21" t="s">
+      <c r="A1" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="F1" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="I1" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="J1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="L1" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="M1" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="O1" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="P1" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q1" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="R1" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="S1" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="T1" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="U1" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="V1" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="W1" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="X1" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="Y1" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="H1" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="I1" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="J1" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="L1" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="M1" s="23" t="s">
+      <c r="Z1" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA1" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB1" s="21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" ht="30" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="N1" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="O1" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="P1" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q1" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="R1" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="S1" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="T1" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="U1" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="V1" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="W1" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="X1" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y1" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="Z1" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA1" s="22" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB1" s="23" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:31" ht="45" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>0</v>
-      </c>
       <c r="C2" s="9" t="s">
-        <v>66</v>
+        <v>16</v>
       </c>
       <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
+      <c r="E2" s="15"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -3978,38 +3957,36 @@
       <c r="N2" s="6"/>
       <c r="O2" s="6"/>
       <c r="P2" s="6"/>
-      <c r="Q2" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
       <c r="T2" s="6"/>
       <c r="U2" s="6"/>
-      <c r="V2" s="16"/>
-      <c r="W2" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="X2" s="16"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="X2" s="5"/>
       <c r="Y2" s="6"/>
       <c r="Z2" s="6"/>
       <c r="AA2" s="6"/>
       <c r="AB2" s="7">
         <f>COUNTA(Table1[[#This Row],[Abstract]:[Zwart-wit]])</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="30" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" ht="52" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="6"/>
-      <c r="E3" s="15"/>
+      <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -4017,103 +3994,105 @@
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
+      <c r="M3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="6"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
       <c r="T3" s="6"/>
       <c r="U3" s="6"/>
       <c r="V3" s="6"/>
-      <c r="W3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="X3" s="5"/>
-      <c r="Y3" s="6"/>
-      <c r="Z3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="Z3" s="5"/>
       <c r="AA3" s="6"/>
       <c r="AB3" s="7">
         <f>COUNTA(Table1[[#This Row],[Abstract]:[Zwart-wit]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="52" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" ht="43" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
+      <c r="G4" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
       <c r="S4" s="6"/>
       <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
-      <c r="V4" s="6"/>
+      <c r="U4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="V4" s="5"/>
       <c r="W4" s="6"/>
       <c r="X4" s="6"/>
-      <c r="Y4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="Z4" s="5"/>
+      <c r="Y4" s="6"/>
+      <c r="Z4" s="6"/>
       <c r="AA4" s="6"/>
       <c r="AB4" s="7">
         <f>COUNTA(Table1[[#This Row],[Abstract]:[Zwart-wit]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:31" ht="43" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" ht="93" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
-      <c r="G5" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="L5" s="15"/>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
+      <c r="R5" s="5"/>
+      <c r="S5" s="5"/>
       <c r="T5" s="6"/>
-      <c r="U5" s="5" t="s">
-        <v>5</v>
-      </c>
+      <c r="U5" s="6"/>
       <c r="V5" s="5"/>
       <c r="W5" s="6"/>
       <c r="X5" s="6"/>
@@ -4125,15 +4104,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:31" ht="93" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" ht="36" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -4141,23 +4120,21 @@
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
-      <c r="J6" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="K6" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="L6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
       <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
       <c r="T6" s="6"/>
-      <c r="U6" s="6"/>
-      <c r="V6" s="5"/>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5" t="s">
+        <v>6</v>
+      </c>
       <c r="W6" s="6"/>
       <c r="X6" s="6"/>
       <c r="Y6" s="6"/>
@@ -4165,40 +4142,40 @@
       <c r="AA6" s="6"/>
       <c r="AB6" s="7">
         <f>COUNTA(Table1[[#This Row],[Abstract]:[Zwart-wit]])</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:31" ht="36" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" ht="62" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="9" t="s">
         <v>24</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
+      <c r="H7" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" s="5"/>
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
       <c r="R7" s="6"/>
       <c r="S7" s="6"/>
       <c r="T7" s="6"/>
-      <c r="U7" s="5"/>
-      <c r="V7" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
       <c r="W7" s="6"/>
       <c r="X7" s="6"/>
       <c r="Y7" s="6"/>
@@ -4209,28 +4186,30 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="62" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" ht="58" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
+      <c r="E8" s="15" t="s">
+        <v>9</v>
+      </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
-      <c r="H8" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="I8" s="5"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
+      <c r="M8" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="N8" s="6"/>
       <c r="O8" s="6"/>
       <c r="P8" s="6"/>
@@ -4244,132 +4223,133 @@
       <c r="X8" s="6"/>
       <c r="Y8" s="6"/>
       <c r="Z8" s="6"/>
-      <c r="AA8" s="6"/>
+      <c r="AA8" s="5"/>
       <c r="AB8" s="7">
         <f>COUNTA(Table1[[#This Row],[Abstract]:[Zwart-wit]])</f>
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AE8" s="17"/>
     </row>
-    <row r="9" spans="1:31" ht="58" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" ht="93" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+        <v>71</v>
+      </c>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="N9" s="6"/>
+      <c r="J9" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="K9" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
       <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
+      <c r="P9" s="22"/>
       <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
-      <c r="T9" s="6"/>
-      <c r="U9" s="6"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="6"/>
-      <c r="X9" s="6"/>
-      <c r="Y9" s="6"/>
+      <c r="R9" s="22"/>
+      <c r="S9" s="22"/>
+      <c r="T9" s="22"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="22"/>
+      <c r="Y9" s="22"/>
       <c r="Z9" s="6"/>
-      <c r="AA9" s="5"/>
+      <c r="AA9" s="22"/>
       <c r="AB9" s="7">
         <f>COUNTA(Table1[[#This Row],[Abstract]:[Zwart-wit]])</f>
         <v>2</v>
       </c>
-      <c r="AE9" s="19"/>
+      <c r="AE9" s="17"/>
     </row>
-    <row r="10" spans="1:31" ht="93" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" ht="39" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
+        <v>29</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="15"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
-      <c r="J10" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="K10" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="L10" s="24"/>
-      <c r="M10" s="24"/>
-      <c r="N10" s="24"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
       <c r="O10" s="6"/>
-      <c r="P10" s="24"/>
+      <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
-      <c r="R10" s="24"/>
-      <c r="S10" s="24"/>
-      <c r="T10" s="24"/>
-      <c r="U10" s="24"/>
-      <c r="V10" s="24"/>
-      <c r="W10" s="24"/>
-      <c r="X10" s="24"/>
-      <c r="Y10" s="24"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+      <c r="U10" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="V10" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="W10" s="6"/>
+      <c r="X10" s="6"/>
+      <c r="Y10" s="6"/>
       <c r="Z10" s="6"/>
-      <c r="AA10" s="24"/>
-      <c r="AB10" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE10" s="19"/>
+      <c r="AA10" s="6"/>
+      <c r="AB10" s="7">
+        <f>COUNTA(Table1[[#This Row],[Abstract]:[Zwart-wit]])</f>
+        <v>2</v>
+      </c>
     </row>
-    <row r="11" spans="1:31" ht="39" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" ht="65" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="15"/>
+        <v>32</v>
+      </c>
+      <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
+      <c r="J11" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
       <c r="M11" s="6"/>
       <c r="N11" s="6"/>
       <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
+      <c r="P11" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q11" s="5"/>
       <c r="R11" s="6"/>
       <c r="S11" s="6"/>
       <c r="T11" s="6"/>
-      <c r="U11" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="V11" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="U11" s="6"/>
+      <c r="V11" s="6"/>
       <c r="W11" s="6"/>
       <c r="X11" s="6"/>
       <c r="Y11" s="6"/>
@@ -4380,58 +4360,52 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:31" ht="65" x14ac:dyDescent="0.3">
-      <c r="A12" s="10" t="s">
-        <v>60</v>
-      </c>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="A12" s="3"/>
       <c r="B12" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="6"/>
+        <v>78</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" s="22"/>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
-      <c r="J12" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
       <c r="M12" s="6"/>
       <c r="N12" s="6"/>
       <c r="O12" s="6"/>
-      <c r="P12" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q12" s="5"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
       <c r="R12" s="6"/>
       <c r="S12" s="6"/>
       <c r="T12" s="6"/>
       <c r="U12" s="6"/>
       <c r="V12" s="6"/>
-      <c r="W12" s="6"/>
-      <c r="X12" s="6"/>
+      <c r="W12" s="5"/>
+      <c r="X12" s="5"/>
       <c r="Y12" s="6"/>
       <c r="Z12" s="6"/>
       <c r="AA12" s="6"/>
       <c r="AB12" s="7">
         <f>COUNTA(Table1[[#This Row],[Abstract]:[Zwart-wit]])</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:31" ht="50" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>34</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>35</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -4444,7 +4418,7 @@
       <c r="L13" s="5"/>
       <c r="M13" s="6"/>
       <c r="N13" s="5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" s="5"/>
       <c r="P13" s="6"/>
@@ -4452,7 +4426,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="6"/>
       <c r="T13" s="5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6"/>
       <c r="V13" s="6"/>
@@ -4468,13 +4442,13 @@
     </row>
     <row r="14" spans="1:31" ht="65" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B14" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>36</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>37</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="15"/>
@@ -4483,12 +4457,12 @@
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="5" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
       <c r="M14" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N14" s="6"/>
       <c r="O14" s="6"/>
@@ -4511,13 +4485,13 @@
     </row>
     <row r="15" spans="1:31" ht="62" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B15" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>39</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>40</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
@@ -4542,7 +4516,7 @@
       <c r="X15" s="6"/>
       <c r="Y15" s="6"/>
       <c r="Z15" s="15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="AA15" s="6"/>
       <c r="AB15" s="7">
@@ -4552,13 +4526,13 @@
     </row>
     <row r="16" spans="1:31" ht="47" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B16" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>41</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>42</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="5"/>
@@ -4573,7 +4547,7 @@
       <c r="N16" s="6"/>
       <c r="O16" s="6"/>
       <c r="P16" s="5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q16" s="5"/>
       <c r="R16" s="6"/>
@@ -4582,7 +4556,7 @@
       <c r="U16" s="6"/>
       <c r="V16" s="6"/>
       <c r="W16" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X16" s="5"/>
       <c r="Y16" s="6"/>
@@ -4595,13 +4569,13 @@
     </row>
     <row r="17" spans="1:28" ht="97" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B17" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="9" t="s">
         <v>43</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>44</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
@@ -4610,14 +4584,14 @@
       <c r="H17" s="6"/>
       <c r="I17" s="6"/>
       <c r="J17" s="5" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
       <c r="M17" s="6"/>
       <c r="N17" s="6"/>
       <c r="O17" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="P17" s="6"/>
       <c r="Q17" s="6"/>
@@ -4625,7 +4599,7 @@
       <c r="S17" s="6"/>
       <c r="T17" s="6"/>
       <c r="U17" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V17" s="6"/>
       <c r="W17" s="6"/>
@@ -4640,16 +4614,16 @@
     </row>
     <row r="18" spans="1:28" ht="45" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B18" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>46</v>
-      </c>
       <c r="D18" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
@@ -4661,7 +4635,7 @@
       <c r="L18" s="6"/>
       <c r="M18" s="5"/>
       <c r="N18" s="5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O18" s="5"/>
       <c r="P18" s="6"/>
@@ -4683,20 +4657,20 @@
     </row>
     <row r="19" spans="1:28" ht="59" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B19" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="9" t="s">
-        <v>48</v>
-      </c>
       <c r="D19" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19" s="6"/>
       <c r="F19" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
@@ -4726,18 +4700,18 @@
     </row>
     <row r="20" spans="1:28" ht="59" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B20" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>49</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>50</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
@@ -4746,7 +4720,7 @@
       <c r="K20" s="6"/>
       <c r="L20" s="6"/>
       <c r="M20" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N20" s="6"/>
       <c r="O20" s="6"/>
@@ -4769,13 +4743,13 @@
     </row>
     <row r="21" spans="1:28" ht="39" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>51</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="15"/>
@@ -4795,7 +4769,7 @@
       <c r="S21" s="6"/>
       <c r="T21" s="6"/>
       <c r="U21" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V21" s="6"/>
       <c r="W21" s="6"/>
@@ -4810,21 +4784,21 @@
     </row>
     <row r="22" spans="1:28" ht="45" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="9" t="s">
-        <v>54</v>
-      </c>
       <c r="D22" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
       <c r="G22" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H22" s="15"/>
       <c r="I22" s="15"/>
@@ -4842,7 +4816,7 @@
       <c r="U22" s="6"/>
       <c r="V22" s="6"/>
       <c r="W22" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X22" s="5"/>
       <c r="Y22" s="6"/>
@@ -4855,13 +4829,13 @@
     </row>
     <row r="23" spans="1:28" ht="39" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B23" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="9" t="s">
         <v>55</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>56</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
@@ -4879,11 +4853,11 @@
       <c r="Q23" s="6"/>
       <c r="R23" s="6"/>
       <c r="S23" s="15" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="T23" s="6"/>
       <c r="U23" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V23" s="6"/>
       <c r="W23" s="5"/>
@@ -4898,13 +4872,13 @@
     </row>
     <row r="24" spans="1:28" ht="52" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="15"/>
@@ -4916,7 +4890,7 @@
       <c r="K24" s="6"/>
       <c r="L24" s="6"/>
       <c r="M24" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N24" s="6"/>
       <c r="O24" s="6"/>
@@ -4930,7 +4904,7 @@
       <c r="W24" s="6"/>
       <c r="X24" s="6"/>
       <c r="Y24" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Z24" s="5"/>
       <c r="AA24" s="6"/>
@@ -4941,13 +4915,13 @@
     </row>
     <row r="25" spans="1:28" ht="39" x14ac:dyDescent="0.3">
       <c r="A25" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B25" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" s="9" t="s">
         <v>58</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>59</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
@@ -4967,10 +4941,10 @@
       <c r="S25" s="6"/>
       <c r="T25" s="6"/>
       <c r="U25" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V25" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W25" s="5"/>
       <c r="X25" s="5"/>
@@ -5084,201 +5058,201 @@
       <c r="AB26" s="7"/>
     </row>
     <row r="27" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="29">
+      <c r="A27" s="23">
         <f>COUNTIF(A2:A25,"✓")/COUNTA(B2:B25)</f>
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="D27" s="11">
+        <f>COUNTA(D2:D25)</f>
+        <v>3</v>
+      </c>
+      <c r="E27" s="11">
+        <f>COUNTA(E2:E25)</f>
         <v>1</v>
       </c>
-      <c r="D27" s="11">
-        <f t="shared" ref="D27:AA27" si="1">COUNTA(D2:D25)</f>
+      <c r="F27" s="11">
+        <f>COUNTA(F2:F25)</f>
+        <v>2</v>
+      </c>
+      <c r="G27" s="11">
+        <f>COUNTA(G2:G25)</f>
+        <v>2</v>
+      </c>
+      <c r="H27" s="11">
+        <f>COUNTA(H2:H25)</f>
+        <v>1</v>
+      </c>
+      <c r="I27" s="11">
+        <f>COUNTA(I2:I25)</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="11">
+        <f>COUNTA(J2:J25)</f>
+        <v>5</v>
+      </c>
+      <c r="K27" s="11">
+        <f>COUNTA(K2:K25)</f>
+        <v>2</v>
+      </c>
+      <c r="L27" s="11">
+        <f>COUNTA(L2:L25)</f>
+        <v>0</v>
+      </c>
+      <c r="M27" s="11">
+        <f>COUNTA(M2:M25)</f>
+        <v>5</v>
+      </c>
+      <c r="N27" s="11">
+        <f>COUNTA(N2:N25)</f>
+        <v>2</v>
+      </c>
+      <c r="O27" s="11">
+        <f>COUNTA(O2:O25)</f>
+        <v>1</v>
+      </c>
+      <c r="P27" s="11">
+        <f>COUNTA(P2:P25)</f>
+        <v>2</v>
+      </c>
+      <c r="Q27" s="11">
+        <f>COUNTA(Q2:Q25)</f>
+        <v>0</v>
+      </c>
+      <c r="R27" s="11">
+        <f>COUNTA(R2:R25)</f>
+        <v>0</v>
+      </c>
+      <c r="S27" s="11">
+        <f>COUNTA(S2:S25)</f>
+        <v>1</v>
+      </c>
+      <c r="T27" s="11">
+        <f>COUNTA(T2:T25)</f>
+        <v>1</v>
+      </c>
+      <c r="U27" s="11">
+        <f>COUNTA(U2:U25)</f>
+        <v>6</v>
+      </c>
+      <c r="V27" s="11">
+        <f>COUNTA(V2:V25)</f>
         <v>3</v>
       </c>
-      <c r="E27" s="11">
-        <f t="shared" si="1"/>
+      <c r="W27" s="11">
+        <f>COUNTA(W2:W25)</f>
+        <v>3</v>
+      </c>
+      <c r="X27" s="11">
+        <f>COUNTA(X2:X25)</f>
+        <v>0</v>
+      </c>
+      <c r="Y27" s="11">
+        <f>COUNTA(Y2:Y25)</f>
+        <v>2</v>
+      </c>
+      <c r="Z27" s="11">
+        <f>COUNTA(Z2:Z25)</f>
         <v>1</v>
       </c>
-      <c r="F27" s="11">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="G27" s="11">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="H27" s="11">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="I27" s="11">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J27" s="11">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K27" s="11">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="L27" s="11">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M27" s="11">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="N27" s="11">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="O27" s="11">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="P27" s="11">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="Q27" s="11">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="R27" s="11">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="S27" s="11">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="T27" s="11">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="U27" s="11">
-        <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="V27" s="11">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="W27" s="11">
-        <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="X27" s="11">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y27" s="11">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="Z27" s="11">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
       <c r="AA27" s="11">
-        <f t="shared" si="1"/>
+        <f>COUNTA(AA2:AA25)</f>
         <v>0</v>
       </c>
       <c r="AB27" s="13">
         <f>SUM(Table1[[#Totals],[Abstract]:[Zwart-wit]])</f>
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A29" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="B29" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
+      <c r="A29" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="26"/>
+      <c r="I29" s="26"/>
+      <c r="J29" s="26"/>
+      <c r="K29" s="26"/>
       <c r="AB29" s="14"/>
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A30" s="27"/>
-      <c r="B30" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="28"/>
-      <c r="K30" s="28"/>
+      <c r="A30" s="25"/>
+      <c r="B30" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A31" s="27"/>
-      <c r="B31" s="28" t="s">
-        <v>78</v>
-      </c>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="28"/>
-      <c r="K31" s="28"/>
+      <c r="A31" s="25"/>
+      <c r="B31" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26"/>
+      <c r="I31" s="26"/>
+      <c r="J31" s="26"/>
+      <c r="K31" s="26"/>
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A32" s="27"/>
-      <c r="B32" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
+      <c r="A32" s="25"/>
+      <c r="B32" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="26"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="26"/>
+      <c r="J32" s="26"/>
+      <c r="K32" s="26"/>
     </row>
     <row r="33" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A33" s="26"/>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="26"/>
-      <c r="K33" s="26"/>
-      <c r="L33" s="26"/>
-      <c r="M33" s="26"/>
-      <c r="N33" s="26"/>
-      <c r="O33" s="26"/>
-      <c r="P33" s="26"/>
-      <c r="Q33" s="26"/>
-      <c r="R33" s="26"/>
-      <c r="S33" s="26"/>
-      <c r="T33" s="26"/>
-      <c r="U33" s="26"/>
-      <c r="V33" s="26"/>
-      <c r="W33" s="26"/>
-      <c r="X33" s="26"/>
-      <c r="Y33" s="26"/>
-      <c r="Z33" s="18"/>
+      <c r="A33" s="24"/>
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="24"/>
+      <c r="K33" s="24"/>
+      <c r="L33" s="24"/>
+      <c r="M33" s="24"/>
+      <c r="N33" s="24"/>
+      <c r="O33" s="24"/>
+      <c r="P33" s="24"/>
+      <c r="Q33" s="24"/>
+      <c r="R33" s="24"/>
+      <c r="S33" s="24"/>
+      <c r="T33" s="24"/>
+      <c r="U33" s="24"/>
+      <c r="V33" s="24"/>
+      <c r="W33" s="24"/>
+      <c r="X33" s="24"/>
+      <c r="Y33" s="24"/>
+      <c r="Z33" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -5300,7 +5274,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB2:AB26">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -5308,7 +5282,7 @@
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="6">
+    <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>